<commit_message>
BOR.OL CR:nc|high. + Excel + D&A
</commit_message>
<xml_diff>
--- a/data/obx_xlsx/BOR.OL.xlsx
+++ b/data/obx_xlsx/BOR.OL.xlsx
@@ -2907,25 +2907,82 @@
       <c r="C30" s="15">
         <v>31.75</v>
       </c>
-      <c r="D30" s="16"/>
-      <c r="E30" s="16"/>
-      <c r="F30" s="16"/>
-      <c r="G30" s="16"/>
-      <c r="H30" s="16"/>
-      <c r="I30" s="16"/>
-      <c r="J30" s="16"/>
-      <c r="K30" s="16"/>
-      <c r="L30" s="16"/>
-      <c r="M30" s="16"/>
-      <c r="N30" s="16"/>
-      <c r="O30" s="16"/>
-      <c r="P30" s="16"/>
-      <c r="Q30" s="16"/>
-      <c r="R30" s="16"/>
-      <c r="S30" s="16"/>
-      <c r="T30" s="16"/>
-      <c r="U30" s="16"/>
-      <c r="V30" s="16"/>
+      <c r="D30" s="16">
+        <f t="shared" ref="D30:V30" si="1">SUM(D31:D37)</f>
+        <v>63.6</v>
+      </c>
+      <c r="E30" s="16">
+        <f t="shared" si="1"/>
+        <v>66.62</v>
+      </c>
+      <c r="F30" s="16">
+        <f t="shared" si="1"/>
+        <v>79.78</v>
+      </c>
+      <c r="G30" s="16">
+        <f t="shared" si="1"/>
+        <v>75.9</v>
+      </c>
+      <c r="H30" s="16">
+        <f t="shared" si="1"/>
+        <v>53.58</v>
+      </c>
+      <c r="I30" s="16">
+        <f t="shared" si="1"/>
+        <v>52.33</v>
+      </c>
+      <c r="J30" s="16">
+        <f t="shared" si="1"/>
+        <v>50.05</v>
+      </c>
+      <c r="K30" s="16">
+        <f t="shared" si="1"/>
+        <v>52.6</v>
+      </c>
+      <c r="L30" s="16">
+        <f t="shared" si="1"/>
+        <v>24.01</v>
+      </c>
+      <c r="M30" s="16">
+        <f t="shared" si="1"/>
+        <v>23.46</v>
+      </c>
+      <c r="N30" s="16">
+        <f t="shared" si="1"/>
+        <v>11.04</v>
+      </c>
+      <c r="O30" s="16">
+        <f t="shared" si="1"/>
+        <v>1.94</v>
+      </c>
+      <c r="P30" s="16">
+        <f t="shared" si="1"/>
+        <v>1.89</v>
+      </c>
+      <c r="Q30" s="16">
+        <f t="shared" si="1"/>
+        <v>1.82</v>
+      </c>
+      <c r="R30" s="16">
+        <f t="shared" si="1"/>
+        <v>1.64</v>
+      </c>
+      <c r="S30" s="16">
+        <f t="shared" si="1"/>
+        <v>1.31</v>
+      </c>
+      <c r="T30" s="16">
+        <f t="shared" si="1"/>
+        <v>27.24</v>
+      </c>
+      <c r="U30" s="16">
+        <f t="shared" si="1"/>
+        <v>53.44</v>
+      </c>
+      <c r="V30" s="16">
+        <f t="shared" si="1"/>
+        <v>48.29</v>
+      </c>
     </row>
     <row r="31" ht="15.0" customHeight="1">
       <c r="A31" s="13" t="s">

</xml_diff>